<commit_message>
added galactic plane, absmag, adjusted plot size
</commit_message>
<xml_diff>
--- a/constellations.xlsx
+++ b/constellations.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twill\Desktop\projects\007_PythonProjects\011_python-snippets\star_plots\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twill\Desktop\projects\007_PythonProjects\constellations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C8637FA-6339-44D4-97AF-0E1F6A3F8A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB3A29EE-9F91-4CB3-9B78-242C26FB14C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25590" yWindow="-15550" windowWidth="25590" windowHeight="21000" activeTab="2" xr2:uid="{B62E7D92-891F-4234-B730-710810B00720}"/>
+    <workbookView xWindow="-216" yWindow="-216" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{B62E7D92-891F-4234-B730-710810B00720}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="const_perim" sheetId="1" r:id="rId1"/>
+    <sheet name="const_areas" sheetId="2" r:id="rId2"/>
+    <sheet name="colors" sheetId="3" r:id="rId3"/>
+    <sheet name="plot_graphs" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3300" uniqueCount="958">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3310" uniqueCount="965">
   <si>
     <t>+34:30:00</t>
   </si>
@@ -2912,6 +2913,27 @@
   </si>
   <si>
     <t xml:space="preserve">	255</t>
+  </si>
+  <si>
+    <t>GLOBE_MAX</t>
+  </si>
+  <si>
+    <t>GLOBE_MIN</t>
+  </si>
+  <si>
+    <t>+2</t>
+  </si>
+  <si>
+    <t>values</t>
+  </si>
+  <si>
+    <t>+8</t>
+  </si>
+  <si>
+    <t>*1</t>
+  </si>
+  <si>
+    <t>*.5</t>
   </si>
 </sst>
 </file>
@@ -2919,9 +2941,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="172" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2931,6 +2953,15 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -2958,7 +2989,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2966,10 +2997,17 @@
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2985,6 +3023,1743 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>plot_graphs!$F$11:$F$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>plot_graphs!$G$11:$G$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.7999999999999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.5999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.3999999999999995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>6.6</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>7.1999999999999993</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>7.8</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>8.4</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>9.6</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>10.199999999999999</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>10.799999999999999</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>11.4</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>12.6</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>13.2</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>13.799999999999999</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>14.399999999999999</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>15.6</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>16.2</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>16.8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-50AF-4FCB-99E9-4257D940A02B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>plot_graphs!$F$11:$F$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>plot_graphs!$H$11:$H$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>0.85555919037101846</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.73198152822831264</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.62625352365755593</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.53579695766745605</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.45840601130522352</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.39219347589350501</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.33554473270424268</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.28707837984570167</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.24561254623381226</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.21013607120076472</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.17978384694427296</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.15381572253342932</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.13159845503703399</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.11259026764556165</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>9.6327638230493035E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>8.2413996174832971E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>7.0510051842580329E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>6.0325522867456564E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>5.1612055503189466E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>4.415716841969286E-2</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>3.7779071262229139E-2</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>3.2322231622081768E-2</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2.7653582317572818E-2</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2.3659276498480913E-2</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2.0241911445804381E-2</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1.7318153368134255E-2</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1.4816705274362072E-2</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1.2676568368499208E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-50AF-4FCB-99E9-4257D940A02B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>plot_graphs!$F$11:$F$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>plot_graphs!$I$11:$I$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>0.85555919037101846</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.73198152822831264</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.62625352365755593</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.53579695766745605</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.45840601130522352</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.39219347589350501</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.33554473270424268</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.28707837984570167</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.24561254623381226</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.21013607120076472</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.17978384694427296</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.15381572253342932</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.13159845503703399</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.11259026764556165</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>9.6327638230493035E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>8.2413996174832971E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>7.0510051842580329E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>6.0325522867456564E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>5.1612055503189466E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>4.415716841969286E-2</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>3.7779071262229139E-2</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>3.2322231622081768E-2</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2.7653582317572818E-2</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2.3659276498480913E-2</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2.0241911445804381E-2</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1.7318153368134255E-2</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1.4816705274362072E-2</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1.2676568368499208E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-50AF-4FCB-99E9-4257D940A02B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>plot_graphs!$F$11:$F$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>plot_graphs!$J$11:$J$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>17.111183807420367</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14.639630564566254</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>12.525070473151118</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10.715939153349121</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9.1681202261044703</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7.8438695178701003</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6.7108946540848535</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.7415675969140336</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4.9122509246762451</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.2027214240152944</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>3.5956769388854593</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3.0763144506685864</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.6319691007406796</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.2518053529112332</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.9265527646098608</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.6482799234966594</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.4102010368516065</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.2065104573491312</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.0322411100637894</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.88314336839385721</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.75558142524458272</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.6464446324416353</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.55307164635145634</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.47318552996961827</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.40483822891608762</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.34636306736268507</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.29633410548724143</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.25353136736998416</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-50AF-4FCB-99E9-4257D940A02B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="293343344"/>
+        <c:axId val="293343704"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="293343344"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="293343704"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="293343704"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="293343344"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>220980</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>41910</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>525780</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>41910</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AFD56062-6B99-8D70-1430-867AF082F4E6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -21557,4 +23332,1404 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A99C71BF-3909-4E79-B052-977A0DC8C8D4}">
+  <dimension ref="E4:J65"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="I4" s="5" t="s">
+        <v>958</v>
+      </c>
+      <c r="J4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="I5" s="5" t="s">
+        <v>959</v>
+      </c>
+      <c r="J5">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="8" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E8" s="5" t="s">
+        <v>961</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>962</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>964</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>960</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="9" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="F9" s="7">
+        <v>8</v>
+      </c>
+      <c r="G9" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="H9" s="7">
+        <v>-0.26</v>
+      </c>
+      <c r="I9" s="7">
+        <v>0</v>
+      </c>
+      <c r="J9" s="7">
+        <f>$J$4</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E10">
+        <v>-8</v>
+      </c>
+      <c r="F10">
+        <f>E10+$F$9</f>
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <f>F10*$G$9</f>
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <f>EXP(G10*$H$9)</f>
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <f>H10+$I$9</f>
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <f>I10*$J$9</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E11">
+        <v>-7</v>
+      </c>
+      <c r="F11">
+        <f t="shared" ref="F11:F38" si="0">E11+$F$9</f>
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <f t="shared" ref="G11:G38" si="1">F11*$G$9</f>
+        <v>0.6</v>
+      </c>
+      <c r="H11">
+        <f t="shared" ref="H11:H38" si="2">EXP(G11*$H$9)</f>
+        <v>0.85555919037101846</v>
+      </c>
+      <c r="I11">
+        <f t="shared" ref="I11:I38" si="3">H11+$I$9</f>
+        <v>0.85555919037101846</v>
+      </c>
+      <c r="J11">
+        <f t="shared" ref="J11:J38" si="4">I11*$J$9</f>
+        <v>17.111183807420367</v>
+      </c>
+    </row>
+    <row r="12" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E12">
+        <v>-6</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="1"/>
+        <v>1.2</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="2"/>
+        <v>0.73198152822831264</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="3"/>
+        <v>0.73198152822831264</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="4"/>
+        <v>14.639630564566254</v>
+      </c>
+    </row>
+    <row r="13" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E13">
+        <v>-5</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="1"/>
+        <v>1.7999999999999998</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="2"/>
+        <v>0.62625352365755593</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="3"/>
+        <v>0.62625352365755593</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="4"/>
+        <v>12.525070473151118</v>
+      </c>
+    </row>
+    <row r="14" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E14">
+        <v>-4</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="1"/>
+        <v>2.4</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="2"/>
+        <v>0.53579695766745605</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="3"/>
+        <v>0.53579695766745605</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="4"/>
+        <v>10.715939153349121</v>
+      </c>
+    </row>
+    <row r="15" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E15">
+        <v>-3</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="2"/>
+        <v>0.45840601130522352</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="3"/>
+        <v>0.45840601130522352</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="4"/>
+        <v>9.1681202261044703</v>
+      </c>
+    </row>
+    <row r="16" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E16">
+        <v>-2</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="1"/>
+        <v>3.5999999999999996</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="2"/>
+        <v>0.39219347589350501</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="3"/>
+        <v>0.39219347589350501</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="4"/>
+        <v>7.8438695178701003</v>
+      </c>
+    </row>
+    <row r="17" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E17">
+        <v>-1</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="1"/>
+        <v>4.2</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="2"/>
+        <v>0.33554473270424268</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="3"/>
+        <v>0.33554473270424268</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="4"/>
+        <v>6.7108946540848535</v>
+      </c>
+    </row>
+    <row r="18" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="1"/>
+        <v>4.8</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="2"/>
+        <v>0.28707837984570167</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="3"/>
+        <v>0.28707837984570167</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="4"/>
+        <v>5.7415675969140336</v>
+      </c>
+    </row>
+    <row r="19" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="1"/>
+        <v>5.3999999999999995</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="2"/>
+        <v>0.24561254623381226</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="3"/>
+        <v>0.24561254623381226</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="4"/>
+        <v>4.9122509246762451</v>
+      </c>
+    </row>
+    <row r="20" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E20">
+        <v>2</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="2"/>
+        <v>0.21013607120076472</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="3"/>
+        <v>0.21013607120076472</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="4"/>
+        <v>4.2027214240152944</v>
+      </c>
+    </row>
+    <row r="21" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E21">
+        <v>3</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="1"/>
+        <v>6.6</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="2"/>
+        <v>0.17978384694427296</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="3"/>
+        <v>0.17978384694427296</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="4"/>
+        <v>3.5956769388854593</v>
+      </c>
+    </row>
+    <row r="22" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E22">
+        <v>4</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="1"/>
+        <v>7.1999999999999993</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="2"/>
+        <v>0.15381572253342932</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="3"/>
+        <v>0.15381572253342932</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="4"/>
+        <v>3.0763144506685864</v>
+      </c>
+    </row>
+    <row r="23" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E23">
+        <v>5</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="1"/>
+        <v>7.8</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="2"/>
+        <v>0.13159845503703399</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="3"/>
+        <v>0.13159845503703399</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="4"/>
+        <v>2.6319691007406796</v>
+      </c>
+    </row>
+    <row r="24" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E24">
+        <v>6</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="1"/>
+        <v>8.4</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="2"/>
+        <v>0.11259026764556165</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="3"/>
+        <v>0.11259026764556165</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="4"/>
+        <v>2.2518053529112332</v>
+      </c>
+    </row>
+    <row r="25" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E25">
+        <v>7</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="2"/>
+        <v>9.6327638230493035E-2</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="3"/>
+        <v>9.6327638230493035E-2</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="4"/>
+        <v>1.9265527646098608</v>
+      </c>
+    </row>
+    <row r="26" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E26">
+        <v>8</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="1"/>
+        <v>9.6</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="2"/>
+        <v>8.2413996174832971E-2</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="3"/>
+        <v>8.2413996174832971E-2</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="4"/>
+        <v>1.6482799234966594</v>
+      </c>
+    </row>
+    <row r="27" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E27">
+        <v>9</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="1"/>
+        <v>10.199999999999999</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="2"/>
+        <v>7.0510051842580329E-2</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="3"/>
+        <v>7.0510051842580329E-2</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="4"/>
+        <v>1.4102010368516065</v>
+      </c>
+    </row>
+    <row r="28" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E28">
+        <v>10</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="1"/>
+        <v>10.799999999999999</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="2"/>
+        <v>6.0325522867456564E-2</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="3"/>
+        <v>6.0325522867456564E-2</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="4"/>
+        <v>1.2065104573491312</v>
+      </c>
+    </row>
+    <row r="29" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E29">
+        <v>11</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="1"/>
+        <v>11.4</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="2"/>
+        <v>5.1612055503189466E-2</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="3"/>
+        <v>5.1612055503189466E-2</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="4"/>
+        <v>1.0322411100637894</v>
+      </c>
+    </row>
+    <row r="30" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E30">
+        <v>12</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="2"/>
+        <v>4.415716841969286E-2</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="3"/>
+        <v>4.415716841969286E-2</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="4"/>
+        <v>0.88314336839385721</v>
+      </c>
+    </row>
+    <row r="31" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E31">
+        <v>13</v>
+      </c>
+      <c r="F31">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="1"/>
+        <v>12.6</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="2"/>
+        <v>3.7779071262229139E-2</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="3"/>
+        <v>3.7779071262229139E-2</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="4"/>
+        <v>0.75558142524458272</v>
+      </c>
+    </row>
+    <row r="32" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E32">
+        <v>14</v>
+      </c>
+      <c r="F32">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="1"/>
+        <v>13.2</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="2"/>
+        <v>3.2322231622081768E-2</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="3"/>
+        <v>3.2322231622081768E-2</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="4"/>
+        <v>0.6464446324416353</v>
+      </c>
+    </row>
+    <row r="33" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E33">
+        <v>15</v>
+      </c>
+      <c r="F33">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="G33">
+        <f t="shared" si="1"/>
+        <v>13.799999999999999</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="2"/>
+        <v>2.7653582317572818E-2</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="3"/>
+        <v>2.7653582317572818E-2</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="4"/>
+        <v>0.55307164635145634</v>
+      </c>
+    </row>
+    <row r="34" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E34">
+        <v>16</v>
+      </c>
+      <c r="F34">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="G34">
+        <f t="shared" si="1"/>
+        <v>14.399999999999999</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="2"/>
+        <v>2.3659276498480913E-2</v>
+      </c>
+      <c r="I34">
+        <f t="shared" si="3"/>
+        <v>2.3659276498480913E-2</v>
+      </c>
+      <c r="J34">
+        <f t="shared" si="4"/>
+        <v>0.47318552996961827</v>
+      </c>
+    </row>
+    <row r="35" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E35">
+        <v>17</v>
+      </c>
+      <c r="F35">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="G35">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="2"/>
+        <v>2.0241911445804381E-2</v>
+      </c>
+      <c r="I35">
+        <f t="shared" si="3"/>
+        <v>2.0241911445804381E-2</v>
+      </c>
+      <c r="J35">
+        <f t="shared" si="4"/>
+        <v>0.40483822891608762</v>
+      </c>
+    </row>
+    <row r="36" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E36">
+        <v>18</v>
+      </c>
+      <c r="F36">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="G36">
+        <f t="shared" si="1"/>
+        <v>15.6</v>
+      </c>
+      <c r="H36">
+        <f t="shared" si="2"/>
+        <v>1.7318153368134255E-2</v>
+      </c>
+      <c r="I36">
+        <f t="shared" si="3"/>
+        <v>1.7318153368134255E-2</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="4"/>
+        <v>0.34636306736268507</v>
+      </c>
+    </row>
+    <row r="37" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E37">
+        <v>19</v>
+      </c>
+      <c r="F37">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="G37">
+        <f t="shared" si="1"/>
+        <v>16.2</v>
+      </c>
+      <c r="H37">
+        <f t="shared" si="2"/>
+        <v>1.4816705274362072E-2</v>
+      </c>
+      <c r="I37">
+        <f t="shared" si="3"/>
+        <v>1.4816705274362072E-2</v>
+      </c>
+      <c r="J37">
+        <f t="shared" si="4"/>
+        <v>0.29633410548724143</v>
+      </c>
+    </row>
+    <row r="38" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E38">
+        <v>20</v>
+      </c>
+      <c r="F38">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="G38">
+        <f t="shared" si="1"/>
+        <v>16.8</v>
+      </c>
+      <c r="H38">
+        <f t="shared" si="2"/>
+        <v>1.2676568368499208E-2</v>
+      </c>
+      <c r="I38">
+        <f t="shared" si="3"/>
+        <v>1.2676568368499208E-2</v>
+      </c>
+      <c r="J38">
+        <f t="shared" si="4"/>
+        <v>0.25353136736998416</v>
+      </c>
+    </row>
+    <row r="41" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E41" s="5" t="s">
+        <v>961</v>
+      </c>
+      <c r="F41" s="6">
+        <v>2</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>963</v>
+      </c>
+      <c r="I41" s="6">
+        <v>0</v>
+      </c>
+      <c r="J41" s="5" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="42" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="F42" s="7">
+        <v>2</v>
+      </c>
+      <c r="G42" s="7">
+        <v>1</v>
+      </c>
+      <c r="H42" s="7">
+        <v>-0.26</v>
+      </c>
+      <c r="I42" s="7">
+        <v>0</v>
+      </c>
+      <c r="J42" s="7">
+        <f>$J$4</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E43">
+        <v>-2</v>
+      </c>
+      <c r="F43">
+        <f>E43+$F$42</f>
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <f>F43*$G$42</f>
+        <v>0</v>
+      </c>
+      <c r="H43">
+        <f t="shared" ref="H43:H65" si="5">EXP(G43*$H$9)</f>
+        <v>1</v>
+      </c>
+      <c r="I43">
+        <f>H43+$I$42</f>
+        <v>1</v>
+      </c>
+      <c r="J43">
+        <f>I43*$J$42</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E44">
+        <v>-1</v>
+      </c>
+      <c r="F44">
+        <f t="shared" ref="F44:F65" si="6">E44+$F$42</f>
+        <v>1</v>
+      </c>
+      <c r="G44">
+        <f t="shared" ref="G44:G65" si="7">F44*$G$42</f>
+        <v>1</v>
+      </c>
+      <c r="H44">
+        <f t="shared" si="5"/>
+        <v>0.77105158580356625</v>
+      </c>
+      <c r="I44">
+        <f t="shared" ref="I44:I65" si="8">H44+$I$42</f>
+        <v>0.77105158580356625</v>
+      </c>
+      <c r="J44">
+        <f t="shared" ref="J44:J65" si="9">I44*$J$42</f>
+        <v>15.421031716071326</v>
+      </c>
+    </row>
+    <row r="45" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="G45">
+        <f t="shared" si="7"/>
+        <v>2</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="5"/>
+        <v>0.59452054797019438</v>
+      </c>
+      <c r="I45">
+        <f t="shared" si="8"/>
+        <v>0.59452054797019438</v>
+      </c>
+      <c r="J45">
+        <f t="shared" si="9"/>
+        <v>11.890410959403887</v>
+      </c>
+    </row>
+    <row r="46" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="G46">
+        <f t="shared" si="7"/>
+        <v>3</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="5"/>
+        <v>0.45840601130522352</v>
+      </c>
+      <c r="I46">
+        <f t="shared" si="8"/>
+        <v>0.45840601130522352</v>
+      </c>
+      <c r="J46">
+        <f t="shared" si="9"/>
+        <v>9.1681202261044703</v>
+      </c>
+    </row>
+    <row r="47" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E47">
+        <v>2</v>
+      </c>
+      <c r="F47">
+        <f t="shared" si="6"/>
+        <v>4</v>
+      </c>
+      <c r="G47">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+      <c r="H47">
+        <f t="shared" si="5"/>
+        <v>0.35345468195878016</v>
+      </c>
+      <c r="I47">
+        <f t="shared" si="8"/>
+        <v>0.35345468195878016</v>
+      </c>
+      <c r="J47">
+        <f t="shared" si="9"/>
+        <v>7.0690936391756036</v>
+      </c>
+    </row>
+    <row r="48" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E48">
+        <v>3</v>
+      </c>
+      <c r="F48">
+        <f t="shared" si="6"/>
+        <v>5</v>
+      </c>
+      <c r="G48">
+        <f t="shared" si="7"/>
+        <v>5</v>
+      </c>
+      <c r="H48">
+        <f t="shared" si="5"/>
+        <v>0.27253179303401259</v>
+      </c>
+      <c r="I48">
+        <f t="shared" si="8"/>
+        <v>0.27253179303401259</v>
+      </c>
+      <c r="J48">
+        <f t="shared" si="9"/>
+        <v>5.4506358606802516</v>
+      </c>
+    </row>
+    <row r="49" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E49">
+        <v>4</v>
+      </c>
+      <c r="F49">
+        <f t="shared" si="6"/>
+        <v>6</v>
+      </c>
+      <c r="G49">
+        <f t="shared" si="7"/>
+        <v>6</v>
+      </c>
+      <c r="H49">
+        <f t="shared" si="5"/>
+        <v>0.21013607120076472</v>
+      </c>
+      <c r="I49">
+        <f t="shared" si="8"/>
+        <v>0.21013607120076472</v>
+      </c>
+      <c r="J49">
+        <f t="shared" si="9"/>
+        <v>4.2027214240152944</v>
+      </c>
+    </row>
+    <row r="50" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E50">
+        <v>5</v>
+      </c>
+      <c r="F50">
+        <f t="shared" si="6"/>
+        <v>7</v>
+      </c>
+      <c r="G50">
+        <f t="shared" si="7"/>
+        <v>7</v>
+      </c>
+      <c r="H50">
+        <f t="shared" si="5"/>
+        <v>0.16202575093388075</v>
+      </c>
+      <c r="I50">
+        <f t="shared" si="8"/>
+        <v>0.16202575093388075</v>
+      </c>
+      <c r="J50">
+        <f t="shared" si="9"/>
+        <v>3.2405150186776148</v>
+      </c>
+    </row>
+    <row r="51" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E51">
+        <v>6</v>
+      </c>
+      <c r="F51">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="G51">
+        <f t="shared" si="7"/>
+        <v>8</v>
+      </c>
+      <c r="H51">
+        <f t="shared" si="5"/>
+        <v>0.12493021219858241</v>
+      </c>
+      <c r="I51">
+        <f t="shared" si="8"/>
+        <v>0.12493021219858241</v>
+      </c>
+      <c r="J51">
+        <f t="shared" si="9"/>
+        <v>2.4986042439716485</v>
+      </c>
+    </row>
+    <row r="52" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E52">
+        <v>7</v>
+      </c>
+      <c r="F52">
+        <f t="shared" si="6"/>
+        <v>9</v>
+      </c>
+      <c r="G52">
+        <f t="shared" si="7"/>
+        <v>9</v>
+      </c>
+      <c r="H52">
+        <f t="shared" si="5"/>
+        <v>9.6327638230493035E-2</v>
+      </c>
+      <c r="I52">
+        <f t="shared" si="8"/>
+        <v>9.6327638230493035E-2</v>
+      </c>
+      <c r="J52">
+        <f t="shared" si="9"/>
+        <v>1.9265527646098608</v>
+      </c>
+    </row>
+    <row r="53" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E53">
+        <v>8</v>
+      </c>
+      <c r="F53">
+        <f t="shared" si="6"/>
+        <v>10</v>
+      </c>
+      <c r="G53">
+        <f t="shared" si="7"/>
+        <v>10</v>
+      </c>
+      <c r="H53">
+        <f t="shared" si="5"/>
+        <v>7.4273578214333877E-2</v>
+      </c>
+      <c r="I53">
+        <f t="shared" si="8"/>
+        <v>7.4273578214333877E-2</v>
+      </c>
+      <c r="J53">
+        <f t="shared" si="9"/>
+        <v>1.4854715642866776</v>
+      </c>
+    </row>
+    <row r="54" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E54">
+        <v>9</v>
+      </c>
+      <c r="F54">
+        <f t="shared" si="6"/>
+        <v>11</v>
+      </c>
+      <c r="G54">
+        <f t="shared" si="7"/>
+        <v>11</v>
+      </c>
+      <c r="H54">
+        <f t="shared" si="5"/>
+        <v>5.7268760265467331E-2</v>
+      </c>
+      <c r="I54">
+        <f t="shared" si="8"/>
+        <v>5.7268760265467331E-2</v>
+      </c>
+      <c r="J54">
+        <f t="shared" si="9"/>
+        <v>1.1453752053093467</v>
+      </c>
+    </row>
+    <row r="55" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E55">
+        <v>10</v>
+      </c>
+      <c r="F55">
+        <f t="shared" si="6"/>
+        <v>12</v>
+      </c>
+      <c r="G55">
+        <f t="shared" si="7"/>
+        <v>12</v>
+      </c>
+      <c r="H55">
+        <f t="shared" si="5"/>
+        <v>4.415716841969286E-2</v>
+      </c>
+      <c r="I55">
+        <f t="shared" si="8"/>
+        <v>4.415716841969286E-2</v>
+      </c>
+      <c r="J55">
+        <f t="shared" si="9"/>
+        <v>0.88314336839385721</v>
+      </c>
+    </row>
+    <row r="56" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E56">
+        <v>11</v>
+      </c>
+      <c r="F56">
+        <f t="shared" si="6"/>
+        <v>13</v>
+      </c>
+      <c r="G56">
+        <f t="shared" si="7"/>
+        <v>13</v>
+      </c>
+      <c r="H56">
+        <f t="shared" si="5"/>
+        <v>3.4047454734599344E-2</v>
+      </c>
+      <c r="I56">
+        <f t="shared" si="8"/>
+        <v>3.4047454734599344E-2</v>
+      </c>
+      <c r="J56">
+        <f t="shared" si="9"/>
+        <v>0.68094909469198694</v>
+      </c>
+    </row>
+    <row r="57" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E57">
+        <v>12</v>
+      </c>
+      <c r="F57">
+        <f t="shared" si="6"/>
+        <v>14</v>
+      </c>
+      <c r="G57">
+        <f t="shared" si="7"/>
+        <v>14</v>
+      </c>
+      <c r="H57">
+        <f t="shared" si="5"/>
+        <v>2.6252343965687961E-2</v>
+      </c>
+      <c r="I57">
+        <f t="shared" si="8"/>
+        <v>2.6252343965687961E-2</v>
+      </c>
+      <c r="J57">
+        <f t="shared" si="9"/>
+        <v>0.52504687931375926</v>
+      </c>
+    </row>
+    <row r="58" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E58">
+        <v>13</v>
+      </c>
+      <c r="F58">
+        <f t="shared" si="6"/>
+        <v>15</v>
+      </c>
+      <c r="G58">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="H58">
+        <f t="shared" si="5"/>
+        <v>2.0241911445804381E-2</v>
+      </c>
+      <c r="I58">
+        <f t="shared" si="8"/>
+        <v>2.0241911445804381E-2</v>
+      </c>
+      <c r="J58">
+        <f t="shared" si="9"/>
+        <v>0.40483822891608762</v>
+      </c>
+    </row>
+    <row r="59" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E59">
+        <v>14</v>
+      </c>
+      <c r="F59">
+        <f t="shared" si="6"/>
+        <v>16</v>
+      </c>
+      <c r="G59">
+        <f t="shared" si="7"/>
+        <v>16</v>
+      </c>
+      <c r="H59">
+        <f t="shared" si="5"/>
+        <v>1.5607557919982831E-2</v>
+      </c>
+      <c r="I59">
+        <f t="shared" si="8"/>
+        <v>1.5607557919982831E-2</v>
+      </c>
+      <c r="J59">
+        <f t="shared" si="9"/>
+        <v>0.31215115839965663</v>
+      </c>
+    </row>
+    <row r="60" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E60">
+        <v>15</v>
+      </c>
+      <c r="F60">
+        <f t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="G60">
+        <f t="shared" si="7"/>
+        <v>17</v>
+      </c>
+      <c r="H60">
+        <f t="shared" si="5"/>
+        <v>1.2034232284723775E-2</v>
+      </c>
+      <c r="I60">
+        <f t="shared" si="8"/>
+        <v>1.2034232284723775E-2</v>
+      </c>
+      <c r="J60">
+        <f t="shared" si="9"/>
+        <v>0.24068464569447551</v>
+      </c>
+    </row>
+    <row r="61" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E61">
+        <v>16</v>
+      </c>
+      <c r="F61">
+        <f t="shared" si="6"/>
+        <v>18</v>
+      </c>
+      <c r="G61">
+        <f t="shared" si="7"/>
+        <v>18</v>
+      </c>
+      <c r="H61">
+        <f t="shared" si="5"/>
+        <v>9.2790138870647437E-3</v>
+      </c>
+      <c r="I61">
+        <f t="shared" si="8"/>
+        <v>9.2790138870647437E-3</v>
+      </c>
+      <c r="J61">
+        <f t="shared" si="9"/>
+        <v>0.18558027774129487</v>
+      </c>
+    </row>
+    <row r="62" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E62">
+        <v>17</v>
+      </c>
+      <c r="F62">
+        <f t="shared" si="6"/>
+        <v>19</v>
+      </c>
+      <c r="G62">
+        <f t="shared" si="7"/>
+        <v>19</v>
+      </c>
+      <c r="H62">
+        <f t="shared" si="5"/>
+        <v>7.1545983723145792E-3</v>
+      </c>
+      <c r="I62">
+        <f t="shared" si="8"/>
+        <v>7.1545983723145792E-3</v>
+      </c>
+      <c r="J62">
+        <f t="shared" si="9"/>
+        <v>0.14309196744629157</v>
+      </c>
+    </row>
+    <row r="63" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E63">
+        <v>18</v>
+      </c>
+      <c r="F63">
+        <f t="shared" si="6"/>
+        <v>20</v>
+      </c>
+      <c r="G63">
+        <f t="shared" si="7"/>
+        <v>20</v>
+      </c>
+      <c r="H63">
+        <f t="shared" si="5"/>
+        <v>5.5165644207607716E-3</v>
+      </c>
+      <c r="I63">
+        <f t="shared" si="8"/>
+        <v>5.5165644207607716E-3</v>
+      </c>
+      <c r="J63">
+        <f t="shared" si="9"/>
+        <v>0.11033128841521543</v>
+      </c>
+    </row>
+    <row r="64" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E64">
+        <v>19</v>
+      </c>
+      <c r="F64">
+        <f t="shared" si="6"/>
+        <v>21</v>
+      </c>
+      <c r="G64">
+        <f t="shared" si="7"/>
+        <v>21</v>
+      </c>
+      <c r="H64">
+        <f t="shared" si="5"/>
+        <v>4.2535557448151254E-3</v>
+      </c>
+      <c r="I64">
+        <f t="shared" si="8"/>
+        <v>4.2535557448151254E-3</v>
+      </c>
+      <c r="J64">
+        <f t="shared" si="9"/>
+        <v>8.5071114896302508E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="5:10" x14ac:dyDescent="0.3">
+      <c r="E65">
+        <v>20</v>
+      </c>
+      <c r="F65">
+        <f t="shared" si="6"/>
+        <v>22</v>
+      </c>
+      <c r="G65">
+        <f t="shared" si="7"/>
+        <v>22</v>
+      </c>
+      <c r="H65">
+        <f t="shared" si="5"/>
+        <v>3.27971090234357E-3</v>
+      </c>
+      <c r="I65">
+        <f t="shared" si="8"/>
+        <v>3.27971090234357E-3</v>
+      </c>
+      <c r="J65">
+        <f t="shared" si="9"/>
+        <v>6.5594218046871405E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>